<commit_message>
Split Wool Tights into Tights and Leggings, adjust all tights to 6-pc packs
Leggings take ~30% of each size's original qty; both halves rounded up
to full 6-piece packs. Bamboo Tights quantities rounded up to packs too.
Tights tab renamed to a general term and Excel export regenerated
(also fixes wrong Wool Socks summary total: 1065 -> 1115 dz).
</commit_message>
<xml_diff>
--- a/public/Roksolana_Order_Aug2026.xlsx
+++ b/public/Roksolana_Order_Aug2026.xlsx
@@ -55,7 +55,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="001a1a2e"/>
+      <color rgb="001A1A2E"/>
       <sz val="8"/>
     </font>
     <font>
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1861,14 +1861,14 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>TIGHTS</t>
+          <t>TIGHTS &amp; LEGGINGS</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>Tights</t>
+          <t>Tights &amp; Leggings</t>
         </is>
       </c>
       <c r="B35" s="30" t="inlineStr">
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="D35" s="18" t="n">
-        <v>120</v>
+        <v>84</v>
       </c>
       <c r="E35" s="17" t="inlineStr">
         <is>
@@ -1909,7 +1909,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Tights</t>
+          <t>Tights &amp; Leggings</t>
         </is>
       </c>
       <c r="B36" s="31" t="inlineStr">
@@ -1923,7 +1923,7 @@
         </is>
       </c>
       <c r="D36" s="7" t="n">
-        <v>180</v>
+        <v>126</v>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t>Tights</t>
+          <t>Tights &amp; Leggings</t>
         </is>
       </c>
       <c r="B37" s="16" t="inlineStr">
@@ -1964,7 +1964,7 @@
         </is>
       </c>
       <c r="D37" s="18" t="n">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="E37" s="17" t="inlineStr">
         <is>
@@ -1991,7 +1991,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Tights</t>
+          <t>Tights &amp; Leggings</t>
         </is>
       </c>
       <c r="B38" s="31" t="inlineStr">
@@ -2005,7 +2005,7 @@
         </is>
       </c>
       <c r="D38" s="7" t="n">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="15" t="inlineStr">
         <is>
-          <t>Tights</t>
+          <t>Tights &amp; Leggings</t>
         </is>
       </c>
       <c r="B39" s="16" t="inlineStr">
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="D39" s="18" t="n">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="E39" s="17" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Tights</t>
+          <t>Tights &amp; Leggings</t>
         </is>
       </c>
       <c r="B40" s="31" t="inlineStr">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="D40" s="7" t="n">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
@@ -2114,12 +2114,12 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t>Tights</t>
+          <t>Tights &amp; Leggings</t>
         </is>
       </c>
       <c r="B41" s="30" t="inlineStr">
         <is>
-          <t>Bamboo Tights</t>
+          <t>Wool Leggings</t>
         </is>
       </c>
       <c r="C41" s="17" t="inlineStr">
@@ -2128,7 +2128,7 @@
         </is>
       </c>
       <c r="D41" s="18" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="E41" s="17" t="inlineStr">
         <is>
@@ -2155,12 +2155,12 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Tights</t>
+          <t>Tights &amp; Leggings</t>
         </is>
       </c>
       <c r="B42" s="31" t="inlineStr">
         <is>
-          <t>Bamboo Tights</t>
+          <t>Wool Leggings</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="D42" s="7" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
@@ -2196,12 +2196,12 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="15" t="inlineStr">
         <is>
-          <t>Tights</t>
+          <t>Tights &amp; Leggings</t>
         </is>
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>Bamboo Tights</t>
+          <t>Wool Leggings</t>
         </is>
       </c>
       <c r="C43" s="17" t="inlineStr">
@@ -2210,7 +2210,7 @@
         </is>
       </c>
       <c r="D43" s="18" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E43" s="17" t="inlineStr">
         <is>
@@ -2237,12 +2237,12 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Tights</t>
+          <t>Tights &amp; Leggings</t>
         </is>
       </c>
       <c r="B44" s="31" t="inlineStr">
         <is>
-          <t>Bamboo Tights</t>
+          <t>Wool Leggings</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="D44" s="7" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
@@ -2278,12 +2278,12 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="15" t="inlineStr">
         <is>
-          <t>Tights</t>
+          <t>Tights &amp; Leggings</t>
         </is>
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>Bamboo Tights</t>
+          <t>Wool Leggings</t>
         </is>
       </c>
       <c r="C45" s="17" t="inlineStr">
@@ -2292,7 +2292,7 @@
         </is>
       </c>
       <c r="D45" s="18" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E45" s="17" t="inlineStr">
         <is>
@@ -2319,12 +2319,12 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Tights</t>
+          <t>Tights &amp; Leggings</t>
         </is>
       </c>
       <c r="B46" s="31" t="inlineStr">
         <is>
-          <t>Bamboo Tights</t>
+          <t>Wool Leggings</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -2333,7 +2333,7 @@
         </is>
       </c>
       <c r="D46" s="7" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
@@ -2357,131 +2357,399 @@
       <c r="L46" s="14" t="n"/>
       <c r="M46" s="14" t="n"/>
     </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>Tights &amp; Leggings</t>
+        </is>
+      </c>
+      <c r="B47" s="30" t="inlineStr">
+        <is>
+          <t>Bamboo Tights</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D47" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="F47" s="19" t="inlineStr">
+        <is>
+          <t>★ NEW</t>
+        </is>
+      </c>
+      <c r="G47" s="20" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="H47" s="33" t="n"/>
+      <c r="I47" s="29" t="n"/>
+      <c r="J47" s="29" t="n"/>
+      <c r="K47" s="29" t="n"/>
+      <c r="L47" s="29" t="n"/>
+      <c r="M47" s="29" t="n"/>
+    </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="39" t="inlineStr">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Tights &amp; Leggings</t>
+        </is>
+      </c>
+      <c r="B48" s="31" t="inlineStr">
+        <is>
+          <t>Bamboo Tights</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>★ NEW</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="H48" s="33" t="n"/>
+      <c r="I48" s="14" t="n"/>
+      <c r="J48" s="14" t="n"/>
+      <c r="K48" s="14" t="n"/>
+      <c r="L48" s="14" t="n"/>
+      <c r="M48" s="14" t="n"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>Tights &amp; Leggings</t>
+        </is>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>Bamboo Tights</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="D49" s="18" t="n">
+        <v>84</v>
+      </c>
+      <c r="E49" s="17" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="F49" s="19" t="inlineStr">
+        <is>
+          <t>★ NEW</t>
+        </is>
+      </c>
+      <c r="G49" s="20" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="H49" s="33" t="n"/>
+      <c r="I49" s="29" t="n"/>
+      <c r="J49" s="29" t="n"/>
+      <c r="K49" s="29" t="n"/>
+      <c r="L49" s="29" t="n"/>
+      <c r="M49" s="29" t="n"/>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Tights &amp; Leggings</t>
+        </is>
+      </c>
+      <c r="B50" s="31" t="inlineStr">
+        <is>
+          <t>Bamboo Tights</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>2XL</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="n">
+        <v>84</v>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>★ NEW</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="H50" s="33" t="n"/>
+      <c r="I50" s="14" t="n"/>
+      <c r="J50" s="14" t="n"/>
+      <c r="K50" s="14" t="n"/>
+      <c r="L50" s="14" t="n"/>
+      <c r="M50" s="14" t="n"/>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="15" t="inlineStr">
+        <is>
+          <t>Tights &amp; Leggings</t>
+        </is>
+      </c>
+      <c r="B51" s="16" t="inlineStr">
+        <is>
+          <t>Bamboo Tights</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="inlineStr">
+        <is>
+          <t>3XL</t>
+        </is>
+      </c>
+      <c r="D51" s="18" t="n">
+        <v>84</v>
+      </c>
+      <c r="E51" s="17" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="F51" s="19" t="inlineStr">
+        <is>
+          <t>★ NEW</t>
+        </is>
+      </c>
+      <c r="G51" s="20" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="H51" s="33" t="n"/>
+      <c r="I51" s="29" t="n"/>
+      <c r="J51" s="29" t="n"/>
+      <c r="K51" s="29" t="n"/>
+      <c r="L51" s="29" t="n"/>
+      <c r="M51" s="29" t="n"/>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Tights &amp; Leggings</t>
+        </is>
+      </c>
+      <c r="B52" s="31" t="inlineStr">
+        <is>
+          <t>Bamboo Tights</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>4XL</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>84</v>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>★ NEW</t>
+        </is>
+      </c>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="H52" s="33" t="n"/>
+      <c r="I52" s="14" t="n"/>
+      <c r="J52" s="14" t="n"/>
+      <c r="K52" s="14" t="n"/>
+      <c r="L52" s="14" t="n"/>
+      <c r="M52" s="14" t="n"/>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="39" t="inlineStr">
         <is>
           <t>ORDER SUMMARY</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="40" t="inlineStr">
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="40" t="inlineStr">
         <is>
           <t>Wool Socks</t>
         </is>
       </c>
-      <c r="B49" s="41" t="n">
-        <v>1065</v>
-      </c>
-      <c r="G49" s="42" t="inlineStr">
-        <is>
-          <t>dz</t>
-        </is>
-      </c>
-      <c r="H49" s="43" t="n"/>
-      <c r="I49" s="43" t="n"/>
-      <c r="J49" s="43" t="n"/>
-      <c r="K49" s="43" t="n"/>
-      <c r="L49" s="43" t="n"/>
-      <c r="M49" s="43" t="n"/>
-    </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="40" t="inlineStr">
+      <c r="B55" s="41" t="n">
+        <v>1115</v>
+      </c>
+      <c r="G55" s="42" t="inlineStr">
+        <is>
+          <t>dz</t>
+        </is>
+      </c>
+      <c r="H55" s="43" t="n"/>
+      <c r="I55" s="43" t="n"/>
+      <c r="J55" s="43" t="n"/>
+      <c r="K55" s="43" t="n"/>
+      <c r="L55" s="43" t="n"/>
+      <c r="M55" s="43" t="n"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="40" t="inlineStr">
         <is>
           <t>Zhytomyr Cotton</t>
         </is>
       </c>
-      <c r="B50" s="41" t="n">
+      <c r="B56" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="G50" s="42" t="inlineStr">
-        <is>
-          <t>dz</t>
-        </is>
-      </c>
-      <c r="H50" s="43" t="n"/>
-      <c r="I50" s="43" t="n"/>
-      <c r="J50" s="43" t="n"/>
-      <c r="K50" s="43" t="n"/>
-      <c r="L50" s="43" t="n"/>
-      <c r="M50" s="43" t="n"/>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="40" t="inlineStr">
+      <c r="G56" s="42" t="inlineStr">
+        <is>
+          <t>dz</t>
+        </is>
+      </c>
+      <c r="H56" s="43" t="n"/>
+      <c r="I56" s="43" t="n"/>
+      <c r="J56" s="43" t="n"/>
+      <c r="K56" s="43" t="n"/>
+      <c r="L56" s="43" t="n"/>
+      <c r="M56" s="43" t="n"/>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="40" t="inlineStr">
         <is>
           <t>Diabetic Socks</t>
         </is>
       </c>
-      <c r="B51" s="41" t="n">
+      <c r="B57" s="41" t="n">
         <v>1550</v>
       </c>
-      <c r="G51" s="42" t="inlineStr">
-        <is>
-          <t>dz</t>
-        </is>
-      </c>
-      <c r="H51" s="43" t="n"/>
-      <c r="I51" s="43" t="n"/>
-      <c r="J51" s="43" t="n"/>
-      <c r="K51" s="43" t="n"/>
-      <c r="L51" s="43" t="n"/>
-      <c r="M51" s="43" t="n"/>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="40" t="inlineStr">
+      <c r="G57" s="42" t="inlineStr">
+        <is>
+          <t>dz</t>
+        </is>
+      </c>
+      <c r="H57" s="43" t="n"/>
+      <c r="I57" s="43" t="n"/>
+      <c r="J57" s="43" t="n"/>
+      <c r="K57" s="43" t="n"/>
+      <c r="L57" s="43" t="n"/>
+      <c r="M57" s="43" t="n"/>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="40" t="inlineStr">
         <is>
           <t>Wool Tights</t>
         </is>
       </c>
-      <c r="B52" s="41" t="n">
-        <v>1300</v>
-      </c>
-      <c r="G52" s="42" t="inlineStr">
+      <c r="B58" s="41" t="n">
+        <v>930</v>
+      </c>
+      <c r="G58" s="42" t="inlineStr">
         <is>
           <t>pcs</t>
         </is>
       </c>
-      <c r="H52" s="43" t="n"/>
-      <c r="I52" s="43" t="n"/>
-      <c r="J52" s="43" t="n"/>
-      <c r="K52" s="43" t="n"/>
-      <c r="L52" s="43" t="n"/>
-      <c r="M52" s="43" t="n"/>
-    </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="40" t="inlineStr">
+      <c r="H58" s="43" t="n"/>
+      <c r="I58" s="43" t="n"/>
+      <c r="J58" s="43" t="n"/>
+      <c r="K58" s="43" t="n"/>
+      <c r="L58" s="43" t="n"/>
+      <c r="M58" s="43" t="n"/>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="40" t="inlineStr">
+        <is>
+          <t>Wool Leggings</t>
+        </is>
+      </c>
+      <c r="B59" s="41" t="n">
+        <v>402</v>
+      </c>
+      <c r="G59" s="42" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="H59" s="43" t="n"/>
+      <c r="I59" s="43" t="n"/>
+      <c r="J59" s="43" t="n"/>
+      <c r="K59" s="43" t="n"/>
+      <c r="L59" s="43" t="n"/>
+      <c r="M59" s="43" t="n"/>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="40" t="inlineStr">
         <is>
           <t>Bamboo Tights</t>
         </is>
       </c>
-      <c r="B53" s="41" t="n">
-        <v>320</v>
-      </c>
-      <c r="G53" s="42" t="inlineStr">
+      <c r="B60" s="41" t="n">
+        <v>420</v>
+      </c>
+      <c r="G60" s="42" t="inlineStr">
         <is>
           <t>pcs</t>
         </is>
       </c>
-      <c r="H53" s="43" t="n"/>
-      <c r="I53" s="43" t="n"/>
-      <c r="J53" s="43" t="n"/>
-      <c r="K53" s="43" t="n"/>
-      <c r="L53" s="43" t="n"/>
-      <c r="M53" s="43" t="n"/>
+      <c r="H60" s="43" t="n"/>
+      <c r="I60" s="43" t="n"/>
+      <c r="J60" s="43" t="n"/>
+      <c r="K60" s="43" t="n"/>
+      <c r="L60" s="43" t="n"/>
+      <c r="M60" s="43" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="B53:F53"/>
+  <mergeCells count="12">
+    <mergeCell ref="B55:F55"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A23:M23"/>
+    <mergeCell ref="B58:F58"/>
     <mergeCell ref="A34:M34"/>
-    <mergeCell ref="B51:F51"/>
-    <mergeCell ref="A48:M48"/>
+    <mergeCell ref="B59:F59"/>
+    <mergeCell ref="B60:F60"/>
     <mergeCell ref="A3:M3"/>
-    <mergeCell ref="B50:F50"/>
     <mergeCell ref="A20:M20"/>
-    <mergeCell ref="B52:F52"/>
-    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="A54:M54"/>
+    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B57:F57"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>

</xml_diff>